<commit_message>
Update master benchmark across 10-fold BioBERT, Sonnet, LLaMA 4 on FAERS and VAERS under Two-Tier Evaluation Framework
</commit_message>
<xml_diff>
--- a/publication/results/comparison_three_schemes/three_schemes_summary.xlsx
+++ b/publication/results/comparison_three_schemes/three_schemes_summary.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,47 +447,32 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>S1 (Relaxed) P</t>
+          <t>Strict P</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S1 (Relaxed) R</t>
+          <t>Strict R</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>S1 (Relaxed) F1</t>
+          <t>Strict F1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>S2 (Weighted) P</t>
+          <t>ADE-Eval P</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>S2 (Weighted) R</t>
+          <t>ADE-Eval R</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>S2 (Weighted) F1</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>S3 (Strict) P</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>S3 (Strict) R</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>S3 (Strict) F1</t>
+          <t>ADE-Eval F1</t>
         </is>
       </c>
     </row>
@@ -499,52 +484,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BioBERT (10-fold)</t>
+          <t>BioBERT (10-fold CV)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9403 +- 0.0056</t>
+          <t>0.6074 +- 0.0207</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.8741 +- 0.0229</t>
+          <t>0.6129 +- 0.0141</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.9058 +- 0.0116</t>
+          <t>0.6099 +- 0.0133</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.8423 +- 0.0103</t>
+          <t>0.8281 +- 0.0101</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.7307 +- 0.0188</t>
+          <t>0.7091 +- 0.0163</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.7824 +- 0.0103</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.6074 +- 0.0207</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0.6759 +- 0.0172</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0.6395 +- 0.0127</t>
+          <t>0.7638 +- 0.0095</t>
         </is>
       </c>
     </row>
@@ -556,52 +526,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claude 4.6 Sonnet</t>
+          <t>Claude 4.6 Sonnet (1-shot)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9106</t>
+          <t>0.4497</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.7802</t>
+          <t>0.4291</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.8404</t>
+          <t>0.4392</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.7500</t>
+          <t>0.7405</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.5647</t>
+          <t>0.5572</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.6443</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.4497</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.4850</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0.4667</t>
+          <t>0.6359</t>
         </is>
       </c>
     </row>
@@ -613,52 +568,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LLaMA 4</t>
+          <t>LLaMA 4 (1-shot)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8648</t>
+          <t>0.3470</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.8476</t>
+          <t>0.4091</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.8561</t>
+          <t>0.3755</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.6778</t>
+          <t>0.6763</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.5796</t>
+          <t>0.5673</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.6249</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.3470</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0.4843</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>0.4043</t>
+          <t>0.6170</t>
         </is>
       </c>
     </row>
@@ -673,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,47 +629,32 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>S1 (Relaxed) P</t>
+          <t>Strict P</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S1 (Relaxed) R</t>
+          <t>Strict R</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>S1 (Relaxed) F1</t>
+          <t>Strict F1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>S2 (Weighted) P</t>
+          <t>ADE-Eval P</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>S2 (Weighted) R</t>
+          <t>ADE-Eval R</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>S2 (Weighted) F1</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>S3 (Strict) P</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>S3 (Strict) R</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>S3 (Strict) F1</t>
+          <t>ADE-Eval F1</t>
         </is>
       </c>
     </row>
@@ -741,52 +666,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BioBERT (10-fold)</t>
+          <t>BioBERT (10-fold CV)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9693 +- 0.0033</t>
+          <t>0.6720 +- 0.0138</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.9282 +- 0.0153</t>
+          <t>0.6185 +- 0.0169</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.9482 +- 0.0076</t>
+          <t>0.6441 +- 0.0136</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.8742 +- 0.0063</t>
+          <t>0.8516 +- 0.0069</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.7481 +- 0.0147</t>
+          <t>0.7177 +- 0.0141</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.8062 +- 0.0094</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.6720 +- 0.0138</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0.7049 +- 0.0141</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0.6880 +- 0.0114</t>
+          <t>0.7789 +- 0.0099</t>
         </is>
       </c>
     </row>
@@ -803,47 +713,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9531</t>
+          <t>0.2949</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.8730</t>
+          <t>0.1973</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.9112</t>
+          <t>0.2364</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.6365</t>
+          <t>0.6448</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.3449</t>
+          <t>0.3780</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.4474</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.2949</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.2509</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0.2711</t>
+          <t>0.4766</t>
         </is>
       </c>
     </row>
@@ -858,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -869,92 +764,62 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision_mean</t>
+          <t>Strict_Precision_mean</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision_std</t>
+          <t>Strict_Precision_std</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall_mean</t>
+          <t>Strict_Recall_mean</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall_std</t>
+          <t>Strict_Recall_std</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1_mean</t>
+          <t>Strict_F1_mean</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1_std</t>
+          <t>Strict_F1_std</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision_mean</t>
+          <t>ADE_Precision_mean</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision_std</t>
+          <t>ADE_Precision_std</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall_mean</t>
+          <t>ADE_Recall_mean</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall_std</t>
+          <t>ADE_Recall_std</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1_mean</t>
+          <t>ADE_F1_mean</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1_std</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision_mean</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision_std</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall_mean</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall_std</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1_mean</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1_std</t>
+          <t>ADE_F1_std</t>
         </is>
       </c>
     </row>
@@ -965,58 +830,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8925999999999999</v>
+        <v>0.5427</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0166</v>
+        <v>0.0359</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8273</v>
+        <v>0.6189</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0516</v>
+        <v>0.0366</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8577</v>
+        <v>0.5772</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0261</v>
+        <v>0.0235</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8142</v>
+        <v>0.8045</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0197</v>
+        <v>0.0193</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7116</v>
+        <v>0.6952</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0405</v>
+        <v>0.0367</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7586000000000001</v>
+        <v>0.7452</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0215</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.5427</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.0359</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.6703</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.0384</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.5985</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.0218</v>
+        <v>0.0203</v>
       </c>
     </row>
     <row r="3">
@@ -1026,58 +873,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9859</v>
+        <v>0.8842</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0064</v>
+        <v>0.034</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9732</v>
+        <v>0.9048</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0185</v>
+        <v>0.0231</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9794</v>
+        <v>0.894</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0073</v>
+        <v>0.0221</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9576</v>
+        <v>0.9534</v>
       </c>
       <c r="I3" t="n">
-        <v>0.012</v>
+        <v>0.0133</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9454</v>
+        <v>0.9368</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0231</v>
+        <v>0.0206</v>
       </c>
       <c r="L3" t="n">
-        <v>0.9513</v>
+        <v>0.9449</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0121</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.8842</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.9225</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.0262</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.9024</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.0203</v>
+        <v>0.0117</v>
       </c>
     </row>
     <row r="4">
@@ -1087,58 +916,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9782</v>
+        <v>0.5332</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0075</v>
+        <v>0.047</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8938</v>
+        <v>0.4919</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0541</v>
+        <v>0.0413</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9332</v>
+        <v>0.5111</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0293</v>
+        <v>0.0404</v>
       </c>
       <c r="H4" t="n">
-        <v>0.785</v>
+        <v>0.773</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0264</v>
+        <v>0.0245</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6926</v>
+        <v>0.6701</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0385</v>
+        <v>0.0353</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7352</v>
+        <v>0.7174</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0247</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.5332</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.047</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.5576</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.0394</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.5444</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.0382</v>
+        <v>0.0244</v>
       </c>
     </row>
     <row r="5">
@@ -1148,58 +959,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.5873</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0137</v>
+        <v>0.0415</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8586</v>
+        <v>0.5929</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0432</v>
+        <v>0.031</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8939</v>
+        <v>0.5889</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0187</v>
+        <v>0.0219</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8358</v>
+        <v>0.8182</v>
       </c>
       <c r="I5" t="n">
-        <v>0.021</v>
+        <v>0.0203</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7167</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0359</v>
+        <v>0.0314</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7708</v>
+        <v>0.7486</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0171</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.5873</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.0415</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.6723</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.0342</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0.6254</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0.0191</v>
+        <v>0.0159</v>
       </c>
     </row>
     <row r="6">
@@ -1209,58 +1002,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9356</v>
+        <v>0.4945</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0132</v>
+        <v>0.0516</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8273</v>
+        <v>0.421</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0679</v>
+        <v>0.0401</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8764</v>
+        <v>0.4522</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0357</v>
+        <v>0.0292</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7846</v>
+        <v>0.7623</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0321</v>
+        <v>0.0293</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5617</v>
+        <v>0.5473</v>
       </c>
       <c r="K6" t="n">
-        <v>0.076</v>
+        <v>0.0603</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6506999999999999</v>
+        <v>0.6344</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0475</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.4945</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.0516</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.5229</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.06759999999999999</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.5032</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.0289</v>
+        <v>0.0376</v>
       </c>
     </row>
     <row r="7">
@@ -1270,58 +1045,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9742</v>
+        <v>0.7067</v>
       </c>
       <c r="C7" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0736</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9189000000000001</v>
+        <v>0.5927</v>
       </c>
       <c r="E7" t="n">
-        <v>0.031</v>
+        <v>0.0473</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9454</v>
+        <v>0.6437</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0152</v>
+        <v>0.0531</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8911</v>
+        <v>0.8672</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0328</v>
+        <v>0.0369</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7017</v>
+        <v>0.6774</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0484</v>
+        <v>0.0416</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7839</v>
+        <v>0.7598</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0302</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.7067</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.0736</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.6719000000000001</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.0433</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.6865</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.0426</v>
+        <v>0.0301</v>
       </c>
     </row>
     <row r="8">
@@ -1331,58 +1088,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4803</v>
+        <v>0.0772</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4417</v>
+        <v>0.1181</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6387</v>
+        <v>0.0226</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1093</v>
+        <v>0.0296</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4299</v>
+        <v>0.0336</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3778</v>
+        <v>0.0446</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1848</v>
+        <v>0.2991</v>
       </c>
       <c r="I8" t="n">
-        <v>0.259</v>
+        <v>0.2711</v>
       </c>
       <c r="J8" t="n">
-        <v>0.0246</v>
+        <v>0.049</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0322</v>
+        <v>0.0501</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0431</v>
+        <v>0.0824</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0565</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.0772</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.1181</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.0246</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.0322</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.0359</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.0478</v>
+        <v>0.0839</v>
       </c>
     </row>
     <row r="9">
@@ -1392,58 +1131,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9643</v>
+        <v>0.5322</v>
       </c>
       <c r="C9" t="n">
-        <v>0.014</v>
+        <v>0.0641</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9038</v>
+        <v>0.5044</v>
       </c>
       <c r="E9" t="n">
-        <v>0.033</v>
+        <v>0.0519</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9326</v>
+        <v>0.5171</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0159</v>
+        <v>0.054</v>
       </c>
       <c r="H9" t="n">
-        <v>0.79</v>
+        <v>0.7759</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0364</v>
+        <v>0.0335</v>
       </c>
       <c r="J9" t="n">
-        <v>0.6927</v>
+        <v>0.6665</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0413</v>
+        <v>0.037</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7375</v>
+        <v>0.7166</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0319</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.5322</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.0641</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.5837</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.5554</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.0526</v>
+        <v>0.0303</v>
       </c>
     </row>
     <row r="10">
@@ -1453,58 +1174,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9695</v>
+        <v>0.8839</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0111</v>
+        <v>0.0376</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9697</v>
+        <v>0.9596</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0235</v>
+        <v>0.0258</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9694</v>
+        <v>0.9194</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0109</v>
+        <v>0.0174</v>
       </c>
       <c r="H10" t="n">
-        <v>0.9671999999999999</v>
+        <v>0.9666</v>
       </c>
       <c r="I10" t="n">
+        <v>0.0113</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.9625</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="M10" t="n">
         <v>0.0112</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.9638</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.0258</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.9653</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.0113</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.8839</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.0376</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.9624</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.9207</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0.0175</v>
       </c>
     </row>
     <row r="11">
@@ -1514,58 +1217,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9085</v>
+        <v>0.6373</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0097</v>
+        <v>0.0337</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8465</v>
+        <v>0.7334000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0368</v>
+        <v>0.0304</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8759</v>
+        <v>0.6811</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0171</v>
+        <v>0.0204</v>
       </c>
       <c r="H11" t="n">
-        <v>0.8662</v>
+        <v>0.8599</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0164</v>
+        <v>0.0175</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7894</v>
+        <v>0.7776999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0389</v>
+        <v>0.0349</v>
       </c>
       <c r="L11" t="n">
-        <v>0.8253</v>
+        <v>0.8161</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0174</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.6373</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.0337</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0.7637</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.0353</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.6936</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.0174</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="12">
@@ -1575,58 +1260,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9802999999999999</v>
+        <v>0.749</v>
       </c>
       <c r="C12" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0545</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9263</v>
+        <v>0.7344000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0376</v>
+        <v>0.0228</v>
       </c>
       <c r="F12" t="n">
-        <v>0.952</v>
+        <v>0.7408</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0174</v>
+        <v>0.0322</v>
       </c>
       <c r="H12" t="n">
-        <v>0.8908</v>
+        <v>0.8862</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0239</v>
+        <v>0.0242</v>
       </c>
       <c r="J12" t="n">
-        <v>0.831</v>
+        <v>0.8223</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0284</v>
+        <v>0.026</v>
       </c>
       <c r="L12" t="n">
-        <v>0.8593</v>
+        <v>0.8526</v>
       </c>
       <c r="M12" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.749</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.0545</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0.754</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.0242</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0.7504</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0.0311</v>
+        <v>0.0135</v>
       </c>
     </row>
   </sheetData>
@@ -1640,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1656,77 +1323,62 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C_boundary</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>C_class</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>C_total</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>S_non_overlap</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>S_wrong_class</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>S_hallucination</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Gold_Total</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Gold_Detected</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision</t>
+          <t>Strict_Precision</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall</t>
+          <t>Strict_Recall</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1</t>
+          <t>Strict_F1</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision</t>
+          <t>ADE_Precision</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall</t>
+          <t>ADE_Recall</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1</t>
+          <t>ADE_F1</t>
         </is>
       </c>
     </row>
@@ -1743,46 +1395,37 @@
         <v>1011</v>
       </c>
       <c r="D2" t="n">
-        <v>3801</v>
+        <v>834</v>
       </c>
       <c r="E2" t="n">
-        <v>834</v>
+        <v>1845</v>
       </c>
       <c r="F2" t="n">
         <v>2740</v>
       </c>
       <c r="G2" t="n">
+        <v>3801</v>
+      </c>
+      <c r="H2" t="n">
         <v>9186</v>
       </c>
-      <c r="H2" t="n">
-        <v>6495</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.9008</v>
+        <v>0.4882</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7071</v>
+        <v>0.4365</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7922</v>
+        <v>0.4609</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7772</v>
+        <v>0.7672</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5312</v>
+        <v>0.5286</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6311</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.4882</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.4762</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.4821</v>
+        <v>0.6259</v>
       </c>
     </row>
     <row r="3">
@@ -1798,46 +1441,37 @@
         <v>35</v>
       </c>
       <c r="D3" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="F3" t="n">
         <v>45</v>
       </c>
       <c r="G3" t="n">
+        <v>59</v>
+      </c>
+      <c r="H3" t="n">
         <v>787</v>
       </c>
-      <c r="H3" t="n">
-        <v>731</v>
-      </c>
       <c r="I3" t="n">
-        <v>0.9848</v>
+        <v>0.8953</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9288</v>
+        <v>0.8794</v>
       </c>
       <c r="K3" t="n">
-        <v>0.956</v>
+        <v>0.8873</v>
       </c>
       <c r="L3" t="n">
-        <v>0.9608</v>
+        <v>0.9605</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9028</v>
+        <v>0.9023</v>
       </c>
       <c r="N3" t="n">
-        <v>0.9308999999999999</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.8953</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.8806</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.8879</v>
+        <v>0.9305</v>
       </c>
     </row>
     <row r="4">
@@ -1853,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="E4" t="n">
         <v>118</v>
@@ -1862,37 +1496,28 @@
         <v>109</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8162</v>
+        <v>0.013</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0.0248</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8988</v>
+        <v>0.0171</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0502</v>
+        <v>0.4182</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>0.5124</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0956</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.0258</v>
+        <v>0.4605</v>
       </c>
     </row>
     <row r="5">
@@ -1908,46 +1533,37 @@
         <v>605</v>
       </c>
       <c r="D5" t="n">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="E5" t="n">
-        <v>225</v>
+        <v>830</v>
       </c>
       <c r="F5" t="n">
         <v>161</v>
       </c>
       <c r="G5" t="n">
+        <v>206</v>
+      </c>
+      <c r="H5" t="n">
         <v>1619</v>
       </c>
-      <c r="H5" t="n">
-        <v>1504</v>
-      </c>
       <c r="I5" t="n">
-        <v>0.976</v>
+        <v>0.4491</v>
       </c>
       <c r="J5" t="n">
-        <v>0.929</v>
+        <v>0.4382</v>
       </c>
       <c r="K5" t="n">
-        <v>0.9519</v>
+        <v>0.4436</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7357</v>
+        <v>0.7287</v>
       </c>
       <c r="M5" t="n">
-        <v>0.6859</v>
+        <v>0.6632</v>
       </c>
       <c r="N5" t="n">
-        <v>0.7099</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.4491</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.4991</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.4728</v>
+        <v>0.6944</v>
       </c>
     </row>
     <row r="6">
@@ -1963,46 +1579,37 @@
         <v>953</v>
       </c>
       <c r="D6" t="n">
-        <v>2458</v>
+        <v>693</v>
       </c>
       <c r="E6" t="n">
-        <v>693</v>
+        <v>1646</v>
       </c>
       <c r="F6" t="n">
         <v>2133</v>
       </c>
       <c r="G6" t="n">
+        <v>2458</v>
+      </c>
+      <c r="H6" t="n">
         <v>6673</v>
       </c>
-      <c r="H6" t="n">
-        <v>5413</v>
-      </c>
       <c r="I6" t="n">
-        <v>0.902</v>
+        <v>0.4633</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8112</v>
+        <v>0.4428</v>
       </c>
       <c r="K6" t="n">
-        <v>0.8542</v>
+        <v>0.4528</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7596000000000001</v>
+        <v>0.7507</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5602</v>
+        <v>0.5546</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6449</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.4633</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.4888</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.4757</v>
+        <v>0.6379</v>
       </c>
     </row>
     <row r="7">
@@ -2018,46 +1625,37 @@
         <v>276</v>
       </c>
       <c r="D7" t="n">
-        <v>760</v>
+        <v>482</v>
       </c>
       <c r="E7" t="n">
-        <v>482</v>
+        <v>758</v>
       </c>
       <c r="F7" t="n">
         <v>579</v>
       </c>
       <c r="G7" t="n">
+        <v>760</v>
+      </c>
+      <c r="H7" t="n">
         <v>1543</v>
       </c>
-      <c r="H7" t="n">
-        <v>1164</v>
-      </c>
       <c r="I7" t="n">
-        <v>0.8973</v>
+        <v>0.2749</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7544</v>
+        <v>0.2504</v>
       </c>
       <c r="K7" t="n">
-        <v>0.8197</v>
+        <v>0.2621</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6153</v>
+        <v>0.6284999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>0.418</v>
+        <v>0.4375</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4978</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.2749</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.3286</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.2994</v>
+        <v>0.5159</v>
       </c>
     </row>
     <row r="8">
@@ -2073,46 +1671,37 @@
         <v>223</v>
       </c>
       <c r="D8" t="n">
-        <v>708</v>
+        <v>157</v>
       </c>
       <c r="E8" t="n">
-        <v>157</v>
+        <v>380</v>
       </c>
       <c r="F8" t="n">
         <v>924</v>
       </c>
       <c r="G8" t="n">
+        <v>708</v>
+      </c>
+      <c r="H8" t="n">
         <v>2408</v>
       </c>
-      <c r="H8" t="n">
-        <v>2091</v>
-      </c>
       <c r="I8" t="n">
-        <v>0.8894</v>
+        <v>0.5311</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8683999999999999</v>
+        <v>0.5758</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8787</v>
+        <v>0.5526</v>
       </c>
       <c r="L8" t="n">
-        <v>0.8062</v>
+        <v>0.7984</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6597</v>
+        <v>0.6499</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7256</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.5311</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.6133999999999999</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.5693</v>
+        <v>0.7165</v>
       </c>
     </row>
     <row r="9">
@@ -2128,46 +1717,37 @@
         <v>21</v>
       </c>
       <c r="D9" t="n">
-        <v>38</v>
+        <v>240</v>
       </c>
       <c r="E9" t="n">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="F9" t="n">
         <v>982</v>
       </c>
       <c r="G9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H9" t="n">
         <v>162</v>
       </c>
-      <c r="H9" t="n">
-        <v>133</v>
-      </c>
       <c r="I9" t="n">
-        <v>0.5972</v>
+        <v>0.0765</v>
       </c>
       <c r="J9" t="n">
-        <v>0.821</v>
+        <v>0.2562</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6914</v>
+        <v>0.1178</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2643</v>
+        <v>0.3831</v>
       </c>
       <c r="M9" t="n">
-        <v>0.7006</v>
+        <v>0.5808</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3838</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.0765</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.6358</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.1366</v>
+        <v>0.4617</v>
       </c>
     </row>
     <row r="10">
@@ -2183,46 +1763,37 @@
         <v>1119</v>
       </c>
       <c r="D10" t="n">
-        <v>989</v>
+        <v>661</v>
       </c>
       <c r="E10" t="n">
-        <v>661</v>
+        <v>1780</v>
       </c>
       <c r="F10" t="n">
         <v>267</v>
       </c>
       <c r="G10" t="n">
+        <v>989</v>
+      </c>
+      <c r="H10" t="n">
         <v>3476</v>
       </c>
-      <c r="H10" t="n">
-        <v>3068</v>
-      </c>
       <c r="I10" t="n">
-        <v>0.9792</v>
+        <v>0.4006</v>
       </c>
       <c r="J10" t="n">
-        <v>0.8826000000000001</v>
+        <v>0.3307</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9284</v>
+        <v>0.3623</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7089</v>
+        <v>0.7024</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5545</v>
+        <v>0.5458</v>
       </c>
       <c r="N10" t="n">
-        <v>0.6223</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.4006</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.3936</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.397</v>
+        <v>0.6143</v>
       </c>
     </row>
     <row r="11">
@@ -2238,46 +1809,37 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>133</v>
       </c>
       <c r="E11" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F11" t="n">
         <v>135</v>
       </c>
       <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
         <v>9</v>
       </c>
-      <c r="H11" t="n">
-        <v>7</v>
-      </c>
       <c r="I11" t="n">
-        <v>0.8046</v>
+        <v>0.0109</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7778</v>
+        <v>0.0211</v>
       </c>
       <c r="K11" t="n">
-        <v>0.791</v>
+        <v>0.0144</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0616</v>
+        <v>0.411</v>
       </c>
       <c r="M11" t="n">
         <v>0.5</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1098</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.0109</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.0212</v>
+        <v>0.4512</v>
       </c>
     </row>
     <row r="12">
@@ -2293,46 +1855,37 @@
         <v>16</v>
       </c>
       <c r="D12" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="F12" t="n">
         <v>94</v>
       </c>
       <c r="G12" t="n">
+        <v>43</v>
+      </c>
+      <c r="H12" t="n">
         <v>767</v>
       </c>
-      <c r="H12" t="n">
-        <v>731</v>
-      </c>
       <c r="I12" t="n">
-        <v>0.9686</v>
+        <v>0.8645</v>
       </c>
       <c r="J12" t="n">
-        <v>0.9530999999999999</v>
+        <v>0.9219000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>0.9608</v>
+        <v>0.8922</v>
       </c>
       <c r="L12" t="n">
-        <v>0.9575</v>
+        <v>0.9572000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>0.9335</v>
+        <v>0.9329</v>
       </c>
       <c r="N12" t="n">
-        <v>0.9454</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.8645</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0.9231</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.8928</v>
+        <v>0.9449</v>
       </c>
     </row>
     <row r="13">
@@ -2348,46 +1901,37 @@
         <v>268</v>
       </c>
       <c r="D13" t="n">
-        <v>1046</v>
+        <v>155</v>
       </c>
       <c r="E13" t="n">
-        <v>155</v>
+        <v>423</v>
       </c>
       <c r="F13" t="n">
         <v>473</v>
       </c>
       <c r="G13" t="n">
+        <v>1046</v>
+      </c>
+      <c r="H13" t="n">
         <v>1796</v>
       </c>
-      <c r="H13" t="n">
-        <v>841</v>
-      </c>
       <c r="I13" t="n">
-        <v>0.8844</v>
+        <v>0.3498</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4683</v>
+        <v>0.2471</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6123</v>
+        <v>0.2896</v>
       </c>
       <c r="L13" t="n">
-        <v>0.6792</v>
+        <v>0.6777</v>
       </c>
       <c r="M13" t="n">
-        <v>0.343</v>
+        <v>0.3555</v>
       </c>
       <c r="N13" t="n">
-        <v>0.4558</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.3498</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.2684</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.3037</v>
+        <v>0.4663</v>
       </c>
     </row>
   </sheetData>
@@ -2401,7 +1945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2417,77 +1961,62 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C_boundary</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>C_class</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>C_total</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>S_non_overlap</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>S_wrong_class</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>S_hallucination</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Gold_Total</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Gold_Detected</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision</t>
+          <t>Strict_Precision</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall</t>
+          <t>Strict_Recall</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1</t>
+          <t>Strict_F1</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision</t>
+          <t>ADE_Precision</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall</t>
+          <t>ADE_Recall</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1</t>
+          <t>ADE_F1</t>
         </is>
       </c>
     </row>
@@ -2504,46 +2033,37 @@
         <v>1301</v>
       </c>
       <c r="D2" t="n">
-        <v>2883</v>
+        <v>971</v>
       </c>
       <c r="E2" t="n">
-        <v>971</v>
+        <v>2272</v>
       </c>
       <c r="F2" t="n">
         <v>5729</v>
       </c>
       <c r="G2" t="n">
+        <v>2883</v>
+      </c>
+      <c r="H2" t="n">
         <v>9186</v>
       </c>
-      <c r="H2" t="n">
-        <v>7490</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.8355</v>
+        <v>0.3847</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8154</v>
+        <v>0.4925</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8253</v>
+        <v>0.432</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7085</v>
+        <v>0.705</v>
       </c>
       <c r="M2" t="n">
-        <v>0.6153</v>
+        <v>0.6042999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6586</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.3847</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.5445</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.4509</v>
+        <v>0.6508</v>
       </c>
     </row>
     <row r="3">
@@ -2559,46 +2079,37 @@
         <v>62</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="F3" t="n">
         <v>119</v>
       </c>
       <c r="G3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H3" t="n">
         <v>787</v>
       </c>
-      <c r="H3" t="n">
-        <v>762</v>
-      </c>
       <c r="I3" t="n">
-        <v>0.9626</v>
+        <v>0.7876</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9681999999999999</v>
+        <v>0.8778</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9654</v>
+        <v>0.8303</v>
       </c>
       <c r="L3" t="n">
-        <v>0.9209000000000001</v>
+        <v>0.9193</v>
       </c>
       <c r="M3" t="n">
-        <v>0.925</v>
+        <v>0.9213</v>
       </c>
       <c r="N3" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.7876</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.8856000000000001</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.8337</v>
+        <v>0.9203</v>
       </c>
     </row>
     <row r="4">
@@ -2614,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>142</v>
       </c>
       <c r="E4" t="n">
         <v>142</v>
@@ -2623,37 +2134,28 @@
         <v>90</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8649</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0.0138</v>
       </c>
       <c r="K4" t="n">
-        <v>0.9275</v>
+        <v>0.0106</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0333</v>
+        <v>0.4384</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6667</v>
+        <v>0.5034</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0635</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.008500000000000001</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.6667</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.0169</v>
+        <v>0.4687</v>
       </c>
     </row>
     <row r="5">
@@ -2669,46 +2171,37 @@
         <v>579</v>
       </c>
       <c r="D5" t="n">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="E5" t="n">
-        <v>287</v>
+        <v>866</v>
       </c>
       <c r="F5" t="n">
         <v>407</v>
       </c>
       <c r="G5" t="n">
+        <v>300</v>
+      </c>
+      <c r="H5" t="n">
         <v>1619</v>
       </c>
-      <c r="H5" t="n">
-        <v>1501</v>
-      </c>
       <c r="I5" t="n">
-        <v>0.9404</v>
+        <v>0.3676</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9271</v>
+        <v>0.3882</v>
       </c>
       <c r="K5" t="n">
-        <v>0.9337</v>
+        <v>0.3776</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6898</v>
+        <v>0.6869</v>
       </c>
       <c r="M5" t="n">
-        <v>0.6359</v>
+        <v>0.6153999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>0.6617</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.3676</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.4571</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.4075</v>
+        <v>0.6492</v>
       </c>
     </row>
     <row r="6">
@@ -2724,46 +2217,37 @@
         <v>1089</v>
       </c>
       <c r="D6" t="n">
-        <v>2174</v>
+        <v>1268</v>
       </c>
       <c r="E6" t="n">
-        <v>1268</v>
+        <v>2357</v>
       </c>
       <c r="F6" t="n">
         <v>4165</v>
       </c>
       <c r="G6" t="n">
+        <v>2174</v>
+      </c>
+      <c r="H6" t="n">
         <v>6673</v>
       </c>
-      <c r="H6" t="n">
-        <v>6431</v>
-      </c>
       <c r="I6" t="n">
-        <v>0.8471</v>
+        <v>0.3433</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9637</v>
+        <v>0.4294</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9016</v>
+        <v>0.3816</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6751</v>
+        <v>0.674</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5926</v>
+        <v>0.5778</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6312</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.3433</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.511</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.4107</v>
+        <v>0.6222</v>
       </c>
     </row>
     <row r="7">
@@ -2779,46 +2263,37 @@
         <v>280</v>
       </c>
       <c r="D7" t="n">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="E7" t="n">
-        <v>744</v>
+        <v>1024</v>
       </c>
       <c r="F7" t="n">
         <v>986</v>
       </c>
       <c r="G7" t="n">
+        <v>740</v>
+      </c>
+      <c r="H7" t="n">
         <v>1543</v>
       </c>
-      <c r="H7" t="n">
-        <v>1227</v>
-      </c>
       <c r="I7" t="n">
-        <v>0.8626</v>
+        <v>0.2065</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7952</v>
+        <v>0.2287</v>
       </c>
       <c r="K7" t="n">
-        <v>0.8275</v>
+        <v>0.217</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5366</v>
+        <v>0.5770999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4297</v>
+        <v>0.4526</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4772</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.2065</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.339</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.2566</v>
+        <v>0.5073</v>
       </c>
     </row>
     <row r="8">
@@ -2834,46 +2309,37 @@
         <v>324</v>
       </c>
       <c r="D8" t="n">
-        <v>728</v>
+        <v>263</v>
       </c>
       <c r="E8" t="n">
-        <v>263</v>
+        <v>587</v>
       </c>
       <c r="F8" t="n">
         <v>1323</v>
       </c>
       <c r="G8" t="n">
+        <v>728</v>
+      </c>
+      <c r="H8" t="n">
         <v>2408</v>
       </c>
-      <c r="H8" t="n">
-        <v>2143</v>
-      </c>
       <c r="I8" t="n">
-        <v>0.8545</v>
+        <v>0.4152</v>
       </c>
       <c r="J8" t="n">
-        <v>0.89</v>
+        <v>0.5077</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8719</v>
+        <v>0.4568</v>
       </c>
       <c r="L8" t="n">
-        <v>0.731</v>
+        <v>0.7255</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6304</v>
+        <v>0.6176</v>
       </c>
       <c r="N8" t="n">
-        <v>0.677</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.4152</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.5631</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.478</v>
+        <v>0.6672</v>
       </c>
     </row>
     <row r="9">
@@ -2889,46 +2355,37 @@
         <v>32</v>
       </c>
       <c r="D9" t="n">
-        <v>33</v>
+        <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>230</v>
+        <v>262</v>
       </c>
       <c r="F9" t="n">
         <v>1056</v>
       </c>
       <c r="G9" t="n">
+        <v>33</v>
+      </c>
+      <c r="H9" t="n">
         <v>162</v>
       </c>
-      <c r="H9" t="n">
-        <v>145</v>
-      </c>
       <c r="I9" t="n">
-        <v>0.5762</v>
+        <v>0.06859999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8951</v>
+        <v>0.2474</v>
       </c>
       <c r="K9" t="n">
-        <v>0.7010999999999999</v>
+        <v>0.1074</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2508</v>
+        <v>0.366</v>
       </c>
       <c r="M9" t="n">
-        <v>0.6975</v>
+        <v>0.5816</v>
       </c>
       <c r="N9" t="n">
-        <v>0.369</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.06859999999999999</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.5988</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.123</v>
+        <v>0.4493</v>
       </c>
     </row>
     <row r="10">
@@ -2944,46 +2401,37 @@
         <v>1570</v>
       </c>
       <c r="D10" t="n">
-        <v>907</v>
+        <v>1154</v>
       </c>
       <c r="E10" t="n">
-        <v>1154</v>
+        <v>2724</v>
       </c>
       <c r="F10" t="n">
         <v>625</v>
       </c>
       <c r="G10" t="n">
+        <v>907</v>
+      </c>
+      <c r="H10" t="n">
         <v>3476</v>
       </c>
-      <c r="H10" t="n">
-        <v>3084</v>
-      </c>
       <c r="I10" t="n">
-        <v>0.9597</v>
+        <v>0.2298</v>
       </c>
       <c r="J10" t="n">
-        <v>0.8872</v>
+        <v>0.2158</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9221</v>
+        <v>0.2225</v>
       </c>
       <c r="L10" t="n">
-        <v>0.592</v>
+        <v>0.6086</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5132</v>
+        <v>0.5099</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5498</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.2298</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.2874</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.2554</v>
+        <v>0.5548999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -2999,46 +2447,37 @@
         <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>85</v>
       </c>
       <c r="E11" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F11" t="n">
         <v>84</v>
       </c>
       <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
         <v>9</v>
       </c>
-      <c r="H11" t="n">
-        <v>7</v>
-      </c>
       <c r="I11" t="n">
-        <v>0.8125</v>
+        <v>0.0057</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7778</v>
+        <v>0.0106</v>
       </c>
       <c r="K11" t="n">
-        <v>0.7948</v>
+        <v>0.0074</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0725</v>
+        <v>0.4107</v>
       </c>
       <c r="M11" t="n">
-        <v>0.3889</v>
+        <v>0.4894</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1223</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.0057</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0.1111</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.0109</v>
+        <v>0.4466</v>
       </c>
     </row>
     <row r="12">
@@ -3054,46 +2493,37 @@
         <v>36</v>
       </c>
       <c r="D12" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="F12" t="n">
         <v>135</v>
       </c>
       <c r="G12" t="n">
+        <v>67</v>
+      </c>
+      <c r="H12" t="n">
         <v>767</v>
       </c>
-      <c r="H12" t="n">
-        <v>719</v>
-      </c>
       <c r="I12" t="n">
-        <v>0.9540999999999999</v>
+        <v>0.7933</v>
       </c>
       <c r="J12" t="n">
-        <v>0.9374</v>
+        <v>0.8635</v>
       </c>
       <c r="K12" t="n">
-        <v>0.9457</v>
+        <v>0.8269</v>
       </c>
       <c r="L12" t="n">
-        <v>0.9288</v>
+        <v>0.9283</v>
       </c>
       <c r="M12" t="n">
-        <v>0.8892</v>
+        <v>0.8882</v>
       </c>
       <c r="N12" t="n">
-        <v>0.9086</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.7933</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0.8657</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.8279</v>
+        <v>0.9078000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -3109,46 +2539,37 @@
         <v>142</v>
       </c>
       <c r="D13" t="n">
-        <v>1377</v>
+        <v>69</v>
       </c>
       <c r="E13" t="n">
-        <v>69</v>
+        <v>211</v>
       </c>
       <c r="F13" t="n">
         <v>550</v>
       </c>
       <c r="G13" t="n">
+        <v>1377</v>
+      </c>
+      <c r="H13" t="n">
         <v>1796</v>
       </c>
-      <c r="H13" t="n">
-        <v>584</v>
-      </c>
       <c r="I13" t="n">
-        <v>0.7802</v>
+        <v>0.2669</v>
       </c>
       <c r="J13" t="n">
-        <v>0.3252</v>
+        <v>0.1485</v>
       </c>
       <c r="K13" t="n">
-        <v>0.459</v>
+        <v>0.1908</v>
       </c>
       <c r="L13" t="n">
-        <v>0.6065</v>
+        <v>0.6115</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1938</v>
+        <v>0.2051</v>
       </c>
       <c r="N13" t="n">
-        <v>0.2937</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.2669</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.1542</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.1955</v>
+        <v>0.3072</v>
       </c>
     </row>
   </sheetData>
@@ -3162,7 +2583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3173,92 +2594,62 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision_mean</t>
+          <t>Strict_Precision_mean</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision_std</t>
+          <t>Strict_Precision_std</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall_mean</t>
+          <t>Strict_Recall_mean</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall_std</t>
+          <t>Strict_Recall_std</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1_mean</t>
+          <t>Strict_F1_mean</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1_std</t>
+          <t>Strict_F1_std</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision_mean</t>
+          <t>ADE_Precision_mean</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision_std</t>
+          <t>ADE_Precision_std</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall_mean</t>
+          <t>ADE_Recall_mean</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall_std</t>
+          <t>ADE_Recall_std</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1_mean</t>
+          <t>ADE_F1_mean</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1_std</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision_mean</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision_std</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall_mean</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall_std</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1_mean</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1_std</t>
+          <t>ADE_F1_std</t>
         </is>
       </c>
     </row>
@@ -3269,58 +2660,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9685</v>
+        <v>0.6173999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0049</v>
+        <v>0.0122</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9204</v>
+        <v>0.5409</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0173</v>
+        <v>0.0178</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9438</v>
+        <v>0.5764</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0094</v>
+        <v>0.0125</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8492</v>
+        <v>0.8221000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>0.006</v>
+        <v>0.0053</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6879</v>
+        <v>0.6581</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0225</v>
+        <v>0.019</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7599</v>
+        <v>0.7309</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0141</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.6173999999999999</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.0122</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.6428</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.0205</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.6297</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.0128</v>
+        <v>0.0124</v>
       </c>
     </row>
     <row r="3">
@@ -3330,58 +2703,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9825</v>
+        <v>0.6766</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0117</v>
+        <v>0.0941</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9348</v>
+        <v>0.5784</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02</v>
+        <v>0.0376</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9579</v>
+        <v>0.6219</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0108</v>
+        <v>0.0559</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8702</v>
+        <v>0.8463000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0403</v>
+        <v>0.0462</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7295</v>
+        <v>0.6928</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0613</v>
+        <v>0.0408</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7912</v>
+        <v>0.7603</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0305</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.6766</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.0941</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.6798</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.0566</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.6721</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.0409</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="4">
@@ -3391,58 +2746,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9427</v>
+        <v>0.5531</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0116</v>
+        <v>0.0474</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8762</v>
+        <v>0.5117</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0306</v>
+        <v>0.0214</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9079</v>
+        <v>0.5305</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0151</v>
+        <v>0.0238</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8113</v>
+        <v>0.7951</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0245</v>
+        <v>0.0257</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6503</v>
+        <v>0.6299</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0436</v>
+        <v>0.0328</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7205</v>
+        <v>0.702</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0203</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.5531</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.0474</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.5865</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.0377</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.5668</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.0172</v>
+        <v>0.0146</v>
       </c>
     </row>
     <row r="5">
@@ -3452,58 +2789,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9536</v>
+        <v>0.665</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0142</v>
+        <v>0.0469</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8974</v>
+        <v>0.6828</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0379</v>
+        <v>0.0273</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9241</v>
+        <v>0.6729000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0183</v>
+        <v>0.0289</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8689</v>
+        <v>0.8549</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0209</v>
+        <v>0.0221</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7984</v>
+        <v>0.7724</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0345</v>
+        <v>0.0271</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8315</v>
+        <v>0.8111</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0168</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.665</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.0469</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.747</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.0344</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0.7020999999999999</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0.0259</v>
+        <v>0.0147</v>
       </c>
     </row>
     <row r="6">
@@ -3513,58 +2832,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9815</v>
+        <v>0.8227</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0054</v>
+        <v>0.036</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9598</v>
+        <v>0.7889</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0129</v>
+        <v>0.0282</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9704</v>
+        <v>0.8052</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0064</v>
+        <v>0.0291</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9346</v>
+        <v>0.9247</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0135</v>
+        <v>0.0159</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8568</v>
+        <v>0.8406</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0211</v>
+        <v>0.0214</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8939</v>
+        <v>0.8804999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0141</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.8227</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.8264</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.0231</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.8242</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.0245</v>
+        <v>0.0161</v>
       </c>
     </row>
     <row r="7">
@@ -3574,58 +2875,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9815</v>
+        <v>0.821</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0053</v>
+        <v>0.0414</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9721</v>
+        <v>0.828</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0135</v>
+        <v>0.0361</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9768</v>
+        <v>0.8243</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0066</v>
+        <v>0.0364</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9238</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0158</v>
+        <v>0.0193</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9052</v>
+        <v>0.8832</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0218</v>
+        <v>0.0234</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9197</v>
+        <v>0.9029</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0155</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.0414</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.8754999999999999</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.8469</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.0293</v>
+        <v>0.0193</v>
       </c>
     </row>
   </sheetData>
@@ -3639,7 +2922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3655,77 +2938,62 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C_boundary</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>C_class</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>C_total</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>S_non_overlap</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>S_wrong_class</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>S_hallucination</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Gold_Total</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Gold_Detected</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>S1_Precision</t>
+          <t>Strict_Precision</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>S1_Recall</t>
+          <t>Strict_Recall</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>S1_F1</t>
+          <t>Strict_F1</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>S2_Precision</t>
+          <t>ADE_Precision</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>S2_Recall</t>
+          <t>ADE_Recall</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>S2_F1</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Precision</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>S3_Recall</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>S3_F1</t>
+          <t>ADE_F1</t>
         </is>
       </c>
     </row>
@@ -3742,46 +3010,37 @@
         <v>3423</v>
       </c>
       <c r="D2" t="n">
-        <v>17160</v>
+        <v>7102</v>
       </c>
       <c r="E2" t="n">
-        <v>7102</v>
+        <v>10525</v>
       </c>
       <c r="F2" t="n">
         <v>1088</v>
       </c>
       <c r="G2" t="n">
+        <v>17160</v>
+      </c>
+      <c r="H2" t="n">
         <v>24087</v>
       </c>
-      <c r="H2" t="n">
-        <v>20711</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.981</v>
+        <v>0.2318</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8598</v>
+        <v>0.1123</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9164</v>
+        <v>0.1513</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5810999999999999</v>
+        <v>0.613</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2165</v>
+        <v>0.2811</v>
       </c>
       <c r="N2" t="n">
-        <v>0.3155</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.2318</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.1455</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.1788</v>
+        <v>0.3854</v>
       </c>
     </row>
     <row r="3">
@@ -3797,46 +3056,37 @@
         <v>548</v>
       </c>
       <c r="D3" t="n">
-        <v>478</v>
+        <v>739</v>
       </c>
       <c r="E3" t="n">
-        <v>739</v>
+        <v>1287</v>
       </c>
       <c r="F3" t="n">
         <v>174</v>
       </c>
       <c r="G3" t="n">
+        <v>478</v>
+      </c>
+      <c r="H3" t="n">
         <v>1378</v>
       </c>
-      <c r="H3" t="n">
-        <v>1216</v>
-      </c>
       <c r="I3" t="n">
-        <v>0.9741</v>
+        <v>0.1942</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8824</v>
+        <v>0.1663</v>
       </c>
       <c r="K3" t="n">
-        <v>0.926</v>
+        <v>0.1791</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5548</v>
+        <v>0.5917</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4543</v>
+        <v>0.4702</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4996</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.1942</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.2554</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.2206</v>
+        <v>0.524</v>
       </c>
     </row>
     <row r="4">
@@ -3852,46 +3102,37 @@
         <v>1201</v>
       </c>
       <c r="D4" t="n">
-        <v>1918</v>
+        <v>1129</v>
       </c>
       <c r="E4" t="n">
-        <v>1129</v>
+        <v>2330</v>
       </c>
       <c r="F4" t="n">
         <v>2062</v>
       </c>
       <c r="G4" t="n">
+        <v>1918</v>
+      </c>
+      <c r="H4" t="n">
         <v>3848</v>
       </c>
-      <c r="H4" t="n">
-        <v>3321</v>
-      </c>
       <c r="I4" t="n">
-        <v>0.8558</v>
+        <v>0.1424</v>
       </c>
       <c r="J4" t="n">
-        <v>0.863</v>
+        <v>0.1465</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8594000000000001</v>
+        <v>0.1444</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4874</v>
+        <v>0.5299</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3455</v>
+        <v>0.3806</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4044</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.1424</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.1894</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.1626</v>
+        <v>0.443</v>
       </c>
     </row>
     <row r="5">
@@ -3907,46 +3148,37 @@
         <v>502</v>
       </c>
       <c r="D5" t="n">
-        <v>564</v>
+        <v>1099</v>
       </c>
       <c r="E5" t="n">
-        <v>1099</v>
+        <v>1601</v>
       </c>
       <c r="F5" t="n">
         <v>542</v>
       </c>
       <c r="G5" t="n">
+        <v>564</v>
+      </c>
+      <c r="H5" t="n">
         <v>1747</v>
       </c>
-      <c r="H5" t="n">
-        <v>1339</v>
-      </c>
       <c r="I5" t="n">
-        <v>0.944</v>
+        <v>0.2411</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7665</v>
+        <v>0.2393</v>
       </c>
       <c r="K5" t="n">
-        <v>0.846</v>
+        <v>0.2402</v>
       </c>
       <c r="L5" t="n">
-        <v>0.585</v>
+        <v>0.6128</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5335</v>
+        <v>0.5206</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5580000000000001</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.2411</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.3898</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.298</v>
+        <v>0.5629</v>
       </c>
     </row>
     <row r="6">
@@ -3962,46 +3194,37 @@
         <v>966</v>
       </c>
       <c r="D6" t="n">
-        <v>1026</v>
+        <v>771</v>
       </c>
       <c r="E6" t="n">
-        <v>771</v>
+        <v>1737</v>
       </c>
       <c r="F6" t="n">
         <v>1100</v>
       </c>
       <c r="G6" t="n">
+        <v>1026</v>
+      </c>
+      <c r="H6" t="n">
         <v>3593</v>
       </c>
-      <c r="H6" t="n">
-        <v>3261</v>
-      </c>
       <c r="I6" t="n">
-        <v>0.9239000000000001</v>
+        <v>0.3607</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9076</v>
+        <v>0.3669</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9157</v>
+        <v>0.3638</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6867</v>
+        <v>0.6835</v>
       </c>
       <c r="M6" t="n">
-        <v>0.58</v>
+        <v>0.5659</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6289</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.3607</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.4456</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.3987</v>
+        <v>0.6192</v>
       </c>
     </row>
     <row r="7">
@@ -4017,46 +3240,37 @@
         <v>968</v>
       </c>
       <c r="D7" t="n">
-        <v>1565</v>
+        <v>159</v>
       </c>
       <c r="E7" t="n">
-        <v>159</v>
+        <v>1127</v>
       </c>
       <c r="F7" t="n">
         <v>700</v>
       </c>
       <c r="G7" t="n">
+        <v>1565</v>
+      </c>
+      <c r="H7" t="n">
         <v>5820</v>
       </c>
-      <c r="H7" t="n">
-        <v>5483</v>
-      </c>
       <c r="I7" t="n">
-        <v>0.9619</v>
+        <v>0.6427</v>
       </c>
       <c r="J7" t="n">
-        <v>0.9421</v>
+        <v>0.5498</v>
       </c>
       <c r="K7" t="n">
-        <v>0.9519</v>
+        <v>0.5926</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8437</v>
+        <v>0.8391</v>
       </c>
       <c r="M7" t="n">
-        <v>0.6479</v>
+        <v>0.644</v>
       </c>
       <c r="N7" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.6427</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.5648</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.6012</v>
+        <v>0.7287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(vaers): update manuscript text, Figure 6, and benchmark tables with new 11-category VAERS results
</commit_message>
<xml_diff>
--- a/publication/results/comparison_three_schemes/three_schemes_summary.xlsx
+++ b/publication/results/comparison_three_schemes/three_schemes_summary.xlsx
@@ -1380,43 +1380,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3504</v>
+        <v>4219</v>
       </c>
       <c r="C2" t="n">
-        <v>3423</v>
+        <v>3632</v>
       </c>
       <c r="D2" t="n">
-        <v>7102</v>
+        <v>6597</v>
       </c>
       <c r="E2" t="n">
-        <v>10525</v>
+        <v>10229</v>
       </c>
       <c r="F2" t="n">
-        <v>1088</v>
+        <v>1235</v>
       </c>
       <c r="G2" t="n">
-        <v>17160</v>
+        <v>16236</v>
       </c>
       <c r="H2" t="n">
         <v>24087</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2318</v>
+        <v>0.269</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1123</v>
+        <v>0.1375</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1513</v>
+        <v>0.182</v>
       </c>
       <c r="L2" t="n">
-        <v>0.613</v>
+        <v>0.6325</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2811</v>
+        <v>0.3042</v>
       </c>
       <c r="N2" t="n">
-        <v>0.3854</v>
+        <v>0.4108</v>
       </c>
     </row>
     <row r="3">
@@ -1426,43 +1426,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="C3" t="n">
-        <v>548</v>
+        <v>614</v>
       </c>
       <c r="D3" t="n">
-        <v>739</v>
+        <v>910</v>
       </c>
       <c r="E3" t="n">
-        <v>1287</v>
+        <v>1524</v>
       </c>
       <c r="F3" t="n">
-        <v>174</v>
+        <v>319</v>
       </c>
       <c r="G3" t="n">
-        <v>478</v>
+        <v>403</v>
       </c>
       <c r="H3" t="n">
         <v>1378</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1942</v>
+        <v>0.1638</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1663</v>
+        <v>0.1578</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1791</v>
+        <v>0.1607</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5917</v>
+        <v>0.5716</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4702</v>
+        <v>0.4908</v>
       </c>
       <c r="N3" t="n">
-        <v>0.524</v>
+        <v>0.5281</v>
       </c>
     </row>
     <row r="4">
@@ -1472,43 +1472,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>729</v>
+        <v>944</v>
       </c>
       <c r="C4" t="n">
-        <v>1201</v>
+        <v>1316</v>
       </c>
       <c r="D4" t="n">
-        <v>1129</v>
+        <v>1049</v>
       </c>
       <c r="E4" t="n">
-        <v>2330</v>
+        <v>2365</v>
       </c>
       <c r="F4" t="n">
-        <v>2062</v>
+        <v>1549</v>
       </c>
       <c r="G4" t="n">
-        <v>1918</v>
+        <v>1588</v>
       </c>
       <c r="H4" t="n">
         <v>3848</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1424</v>
+        <v>0.1943</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1465</v>
+        <v>0.1928</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1444</v>
+        <v>0.1935</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5299</v>
+        <v>0.5753</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3806</v>
+        <v>0.4342</v>
       </c>
       <c r="N4" t="n">
-        <v>0.443</v>
+        <v>0.4949</v>
       </c>
     </row>
     <row r="5">
@@ -1518,43 +1518,43 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>681</v>
+        <v>774</v>
       </c>
       <c r="C5" t="n">
-        <v>502</v>
+        <v>515</v>
       </c>
       <c r="D5" t="n">
-        <v>1099</v>
+        <v>962</v>
       </c>
       <c r="E5" t="n">
-        <v>1601</v>
+        <v>1477</v>
       </c>
       <c r="F5" t="n">
-        <v>542</v>
+        <v>647</v>
       </c>
       <c r="G5" t="n">
-        <v>564</v>
+        <v>458</v>
       </c>
       <c r="H5" t="n">
         <v>1747</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2411</v>
+        <v>0.2671</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2393</v>
+        <v>0.2857</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2402</v>
+        <v>0.2761</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6128</v>
+        <v>0.6269</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5206</v>
+        <v>0.5583</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5629</v>
+        <v>0.5906</v>
       </c>
     </row>
     <row r="6">
@@ -1564,43 +1564,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1601</v>
+        <v>2052</v>
       </c>
       <c r="C6" t="n">
-        <v>966</v>
+        <v>829</v>
       </c>
       <c r="D6" t="n">
-        <v>771</v>
+        <v>417</v>
       </c>
       <c r="E6" t="n">
-        <v>1737</v>
+        <v>1246</v>
       </c>
       <c r="F6" t="n">
-        <v>1100</v>
+        <v>657</v>
       </c>
       <c r="G6" t="n">
-        <v>1026</v>
+        <v>712</v>
       </c>
       <c r="H6" t="n">
         <v>3593</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3607</v>
+        <v>0.5188</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3669</v>
+        <v>0.5117</v>
       </c>
       <c r="K6" t="n">
-        <v>0.3638</v>
+        <v>0.5153</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6835</v>
+        <v>0.7726</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5659</v>
+        <v>0.6671</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6192</v>
+        <v>0.716</v>
       </c>
     </row>
     <row r="7">
@@ -1610,43 +1610,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3287</v>
+        <v>3621</v>
       </c>
       <c r="C7" t="n">
-        <v>968</v>
+        <v>813</v>
       </c>
       <c r="D7" t="n">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="E7" t="n">
-        <v>1127</v>
+        <v>962</v>
       </c>
       <c r="F7" t="n">
-        <v>700</v>
+        <v>846</v>
       </c>
       <c r="G7" t="n">
-        <v>1565</v>
+        <v>1386</v>
       </c>
       <c r="H7" t="n">
         <v>5820</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6427</v>
+        <v>0.667</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5498</v>
+        <v>0.6066</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5926</v>
+        <v>0.6354</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8391</v>
+        <v>0.8556</v>
       </c>
       <c r="M7" t="n">
-        <v>0.644</v>
+        <v>0.6872</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7287</v>
+        <v>0.7622</v>
       </c>
     </row>
   </sheetData>
@@ -2440,32 +2440,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.2949</t>
+          <t>0.3418</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.1973</t>
+          <t>0.2368</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.2364</t>
+          <t>0.2797</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.6448</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.3780</t>
+          <t>0.4129</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.4766</t>
+          <t>0.5113</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align VAERS evaluation metrics to FAERS 1-to-1 standard and update tables, Figure 6, and manuscript
</commit_message>
<xml_diff>
--- a/publication/results/comparison_three_schemes/three_schemes_summary.xlsx
+++ b/publication/results/comparison_three_schemes/three_schemes_summary.xlsx
@@ -1298,7 +1298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1314,60 +1314,55 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>C_boundary</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>C_class</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>C_total</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>S_non_overlap</t>
+          <t>Gold_Total</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Pred_Total</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Gold_Total</t>
+          <t>Strict_Precision</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Strict_Precision</t>
+          <t>Strict_Recall</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Strict_Recall</t>
+          <t>Strict_F1</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Strict_F1</t>
+          <t>ADE_Precision</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>ADE_Precision</t>
+          <t>ADE_Recall</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>ADE_Recall</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ADE_F1</t>
         </is>
@@ -1376,277 +1371,474 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>VAX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4219</v>
+        <v>3615</v>
       </c>
       <c r="C2" t="n">
-        <v>3632</v>
+        <v>1332</v>
       </c>
       <c r="D2" t="n">
-        <v>6597</v>
+        <v>482</v>
       </c>
       <c r="E2" t="n">
-        <v>10229</v>
+        <v>88</v>
       </c>
       <c r="F2" t="n">
-        <v>1235</v>
+        <v>5823</v>
       </c>
       <c r="G2" t="n">
-        <v>16236</v>
+        <v>5429</v>
       </c>
       <c r="H2" t="n">
-        <v>24087</v>
+        <v>0.6659</v>
       </c>
       <c r="I2" t="n">
-        <v>0.269</v>
+        <v>0.718</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1375</v>
+        <v>0.6909</v>
       </c>
       <c r="K2" t="n">
-        <v>0.182</v>
+        <v>0.8448</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6325</v>
+        <v>0.8502</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3042</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.4108</v>
+        <v>0.8475</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HX</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>361</v>
+        <v>2000</v>
       </c>
       <c r="C3" t="n">
-        <v>614</v>
+        <v>1394</v>
       </c>
       <c r="D3" t="n">
-        <v>910</v>
+        <v>561</v>
       </c>
       <c r="E3" t="n">
-        <v>1524</v>
+        <v>146</v>
       </c>
       <c r="F3" t="n">
-        <v>319</v>
+        <v>3607</v>
       </c>
       <c r="G3" t="n">
-        <v>403</v>
+        <v>3955</v>
       </c>
       <c r="H3" t="n">
-        <v>1378</v>
+        <v>0.5057</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1638</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1578</v>
+        <v>0.5337</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1607</v>
+        <v>0.7631</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5716</v>
+        <v>0.7619</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4908</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.5281</v>
+        <v>0.7625</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LAB</t>
+          <t>STATUS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>944</v>
+        <v>776</v>
       </c>
       <c r="C4" t="n">
-        <v>1316</v>
+        <v>1521</v>
       </c>
       <c r="D4" t="n">
-        <v>1049</v>
+        <v>601</v>
       </c>
       <c r="E4" t="n">
-        <v>2365</v>
+        <v>309</v>
       </c>
       <c r="F4" t="n">
-        <v>1549</v>
+        <v>1747</v>
       </c>
       <c r="G4" t="n">
-        <v>1588</v>
+        <v>2898</v>
       </c>
       <c r="H4" t="n">
-        <v>3848</v>
+        <v>0.2678</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1943</v>
+        <v>0.2978</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1928</v>
+        <v>0.282</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1935</v>
+        <v>0.6278</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5753</v>
+        <v>0.5896</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4342</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.4949</v>
+        <v>0.6081</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>MHx</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>774</v>
+        <v>344</v>
       </c>
       <c r="C5" t="n">
-        <v>515</v>
+        <v>1465</v>
       </c>
       <c r="D5" t="n">
-        <v>962</v>
+        <v>197</v>
       </c>
       <c r="E5" t="n">
-        <v>1477</v>
+        <v>68</v>
       </c>
       <c r="F5" t="n">
-        <v>647</v>
+        <v>1183</v>
       </c>
       <c r="G5" t="n">
-        <v>458</v>
+        <v>2006</v>
       </c>
       <c r="H5" t="n">
-        <v>1747</v>
+        <v>0.1715</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2671</v>
+        <v>0.1833</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2857</v>
+        <v>0.1772</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2761</v>
+        <v>0.5793</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6269</v>
+        <v>0.5735</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5583</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.5906</v>
+        <v>0.5764</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>sDx</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2052</v>
+        <v>775</v>
       </c>
       <c r="C6" t="n">
-        <v>829</v>
+        <v>1911</v>
       </c>
       <c r="D6" t="n">
-        <v>417</v>
+        <v>98</v>
       </c>
       <c r="E6" t="n">
-        <v>1246</v>
+        <v>191</v>
       </c>
       <c r="F6" t="n">
-        <v>657</v>
+        <v>8265</v>
       </c>
       <c r="G6" t="n">
-        <v>712</v>
+        <v>2784</v>
       </c>
       <c r="H6" t="n">
-        <v>3593</v>
+        <v>0.2784</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5188</v>
+        <v>0.2694</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5117</v>
+        <v>0.2738</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5153</v>
+        <v>0.6384</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7726</v>
+        <v>0.6015</v>
       </c>
       <c r="M6" t="n">
-        <v>0.6671</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.716</v>
+        <v>0.6194</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VAX</t>
+          <t>pDx</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3621</v>
+        <v>496</v>
       </c>
       <c r="C7" t="n">
-        <v>813</v>
+        <v>689</v>
       </c>
       <c r="D7" t="n">
-        <v>149</v>
+        <v>58</v>
       </c>
       <c r="E7" t="n">
-        <v>962</v>
+        <v>29</v>
       </c>
       <c r="F7" t="n">
-        <v>846</v>
+        <v>1244</v>
       </c>
       <c r="G7" t="n">
-        <v>1386</v>
+        <v>1243</v>
       </c>
       <c r="H7" t="n">
-        <v>5820</v>
+        <v>0.399</v>
       </c>
       <c r="I7" t="n">
-        <v>0.667</v>
+        <v>0.4086</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6066</v>
+        <v>0.4037</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6354</v>
+        <v>0.7007</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8556</v>
+        <v>0.6923</v>
       </c>
       <c r="M7" t="n">
-        <v>0.6872</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.7622</v>
+        <v>0.6965</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SYM</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2984</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8075</v>
+      </c>
+      <c r="D8" t="n">
+        <v>597</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2541</v>
+      </c>
+      <c r="F8" t="n">
+        <v>14581</v>
+      </c>
+      <c r="G8" t="n">
+        <v>11656</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.2194</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.2363</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.6264999999999999</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.5163</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.5661</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>951</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2496</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1411</v>
+      </c>
+      <c r="E9" t="n">
+        <v>567</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3849</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4858</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.1958</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.2369</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.2144</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.5787</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.5478</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.5629</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FHx</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" t="n">
+        <v>159</v>
+      </c>
+      <c r="D10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" t="n">
+        <v>195</v>
+      </c>
+      <c r="G10" t="n">
+        <v>198</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.09089999999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0914</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.0911</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.4949</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.5142</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>15</v>
+      </c>
+      <c r="C11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>46</v>
+      </c>
+      <c r="G11" t="n">
+        <v>45</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.7333</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.6984</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>41</v>
+      </c>
+      <c r="C12" t="n">
+        <v>420</v>
+      </c>
+      <c r="D12" t="n">
+        <v>37</v>
+      </c>
+      <c r="E12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F12" t="n">
+        <v>171</v>
+      </c>
+      <c r="G12" t="n">
+        <v>498</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.0823</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0867</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.0844</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.5338000000000001</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.5306999999999999</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.5322</v>
       </c>
     </row>
   </sheetData>
@@ -2361,27 +2553,27 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.6268 +- 0.0203</t>
+          <t>0.7076 +- 0.0164</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.6594 +- 0.0196</t>
+          <t>0.7015 +- 0.0174</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.8619 +- 0.0095</t>
+          <t>0.8618 +- 0.0096</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.7205 +- 0.0153</t>
+          <t>0.8135 +- 0.0119</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.7848 +- 0.0127</t>
+          <t>0.8370 +- 0.0095</t>
         </is>
       </c>
     </row>
@@ -2403,12 +2595,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.6324 +- 0.0183</t>
+          <t>0.7132 +- 0.0157</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.6595 +- 0.0177</t>
+          <t>0.7009 +- 0.0163</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2418,12 +2610,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.7279 +- 0.0139</t>
+          <t>0.8209 +- 0.0118</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.7882 +- 0.0112</t>
+          <t>0.8397 +- 0.0089</t>
         </is>
       </c>
     </row>
@@ -2435,37 +2627,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LLaMA 4 (1-shot, Target Filtered)</t>
+          <t>LLaMA 4 (1-shot, Tagged)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.3418</t>
+          <t>0.3378</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.2368</t>
+          <t>0.3388</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.2797</t>
+          <t>0.3383</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.6714</t>
+          <t>0.6691</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.4129</t>
+          <t>0.6134</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.5113</t>
+          <t>0.6400</t>
         </is>
       </c>
     </row>
@@ -2792,33 +2984,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>fold</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>C_boundary</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>C_class</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>C_total</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>S_non_overlap</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2828,59 +3020,44 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Total_Gold</t>
+          <t>Strict_Precision</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Strict_Precision</t>
+          <t>Strict_Recall</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Strict_Recall</t>
+          <t>Strict_F1</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Strict_F1</t>
+          <t>ADE_Precision</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>ADE_Precision</t>
+          <t>ADE_Recall</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>ADE_Recall</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>ADE_F1</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>fold</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>seed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C2" t="n">
         <v>1351</v>
-      </c>
-      <c r="B2" t="n">
-        <v>157</v>
-      </c>
-      <c r="C2" t="n">
-        <v>280</v>
       </c>
       <c r="D2" t="n">
         <v>437</v>
@@ -2889,45 +3066,36 @@
         <v>203</v>
       </c>
       <c r="F2" t="n">
-        <v>468</v>
+        <v>193</v>
       </c>
       <c r="G2" t="n">
-        <v>1976</v>
+        <v>0.6785534907081868</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6786</v>
+        <v>0.6819787985865724</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5988</v>
+        <v>0.6802618328298086</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6362</v>
+        <v>0.8535690006798097</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8536</v>
+        <v>0.7922766279656739</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6957</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.7665999999999999</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>42</v>
+        <v>0.8217815302048563</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>42</v>
+      </c>
+      <c r="C3" t="n">
         <v>1585</v>
-      </c>
-      <c r="B3" t="n">
-        <v>191</v>
-      </c>
-      <c r="C3" t="n">
-        <v>329</v>
       </c>
       <c r="D3" t="n">
         <v>520</v>
@@ -2936,45 +3104,36 @@
         <v>183</v>
       </c>
       <c r="F3" t="n">
-        <v>475</v>
+        <v>157</v>
       </c>
       <c r="G3" t="n">
-        <v>2251</v>
+        <v>0.6927447552447552</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6927</v>
+        <v>0.7007073386383731</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6143</v>
+        <v>0.6967032967032967</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6512</v>
+        <v>0.8578402882715331</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8578</v>
+        <v>0.8156498673740054</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7151</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" t="n">
-        <v>42</v>
+        <v>0.8362132457084586</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>42</v>
+      </c>
+      <c r="C4" t="n">
         <v>1484</v>
-      </c>
-      <c r="B4" t="n">
-        <v>190</v>
-      </c>
-      <c r="C4" t="n">
-        <v>296</v>
       </c>
       <c r="D4" t="n">
         <v>486</v>
@@ -2983,45 +3142,36 @@
         <v>200</v>
       </c>
       <c r="F4" t="n">
-        <v>445</v>
+        <v>152</v>
       </c>
       <c r="G4" t="n">
-        <v>2119</v>
+        <v>0.6838709677419355</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6839</v>
+        <v>0.6993402450518379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6145</v>
+        <v>0.6915191053122087</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6473</v>
+        <v>0.8549504950495049</v>
       </c>
       <c r="K4" t="n">
-        <v>0.855</v>
+        <v>0.8138548539114043</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7151</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.7788</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" t="n">
-        <v>42</v>
+        <v>0.833896668276195</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
+        <v>42</v>
+      </c>
+      <c r="C5" t="n">
         <v>1485</v>
-      </c>
-      <c r="B5" t="n">
-        <v>171</v>
-      </c>
-      <c r="C5" t="n">
-        <v>250</v>
       </c>
       <c r="D5" t="n">
         <v>421</v>
@@ -3030,45 +3180,36 @@
         <v>241</v>
       </c>
       <c r="F5" t="n">
-        <v>407</v>
+        <v>160</v>
       </c>
       <c r="G5" t="n">
-        <v>2063</v>
+        <v>0.6916627852817886</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6917</v>
+        <v>0.7187802516940949</v>
       </c>
       <c r="I5" t="n">
-        <v>0.642</v>
+        <v>0.7049608355091384</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6659</v>
+        <v>0.8623013350286077</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8623</v>
+        <v>0.8206679574056147</v>
       </c>
       <c r="L5" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.7924</v>
-      </c>
-      <c r="N5" t="n">
-        <v>3</v>
-      </c>
-      <c r="O5" t="n">
-        <v>42</v>
+        <v>0.8409696819393638</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>42</v>
+      </c>
+      <c r="C6" t="n">
         <v>1565</v>
-      </c>
-      <c r="B6" t="n">
-        <v>168</v>
-      </c>
-      <c r="C6" t="n">
-        <v>241</v>
       </c>
       <c r="D6" t="n">
         <v>409</v>
@@ -3077,45 +3218,36 @@
         <v>201</v>
       </c>
       <c r="F6" t="n">
-        <v>426</v>
+        <v>179</v>
       </c>
       <c r="G6" t="n">
-        <v>2159</v>
+        <v>0.7195402298850575</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7195</v>
+        <v>0.7268927078495123</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6521</v>
+        <v>0.7231977818853975</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6842</v>
+        <v>0.874150920093862</v>
       </c>
       <c r="K6" t="n">
-        <v>0.8742</v>
+        <v>0.8218764514630748</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7373</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.7999000000000001</v>
-      </c>
-      <c r="N6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O6" t="n">
-        <v>42</v>
+        <v>0.8472080914477228</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" t="n">
         <v>1578</v>
-      </c>
-      <c r="B7" t="n">
-        <v>173</v>
-      </c>
-      <c r="C7" t="n">
-        <v>287</v>
       </c>
       <c r="D7" t="n">
         <v>460</v>
@@ -3124,45 +3256,36 @@
         <v>205</v>
       </c>
       <c r="F7" t="n">
-        <v>448</v>
+        <v>166</v>
       </c>
       <c r="G7" t="n">
-        <v>2199</v>
+        <v>0.7035220686580472</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7035</v>
+        <v>0.7159709618874773</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6348</v>
+        <v>0.7096919271418934</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6674</v>
+        <v>0.8653823142275936</v>
       </c>
       <c r="K7" t="n">
-        <v>0.8653999999999999</v>
+        <v>0.8203266787658802</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7272999999999999</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.7903</v>
-      </c>
-      <c r="N7" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" t="n">
-        <v>42</v>
+        <v>0.8422523729109649</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>42</v>
+      </c>
+      <c r="C8" t="n">
         <v>1415</v>
-      </c>
-      <c r="B8" t="n">
-        <v>153</v>
-      </c>
-      <c r="C8" t="n">
-        <v>328</v>
       </c>
       <c r="D8" t="n">
         <v>481</v>
@@ -3171,45 +3294,36 @@
         <v>242</v>
       </c>
       <c r="F8" t="n">
-        <v>454</v>
+        <v>141</v>
       </c>
       <c r="G8" t="n">
-        <v>2022</v>
+        <v>0.6618334892422825</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.6946489936180658</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6021</v>
+        <v>0.6778443113772454</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6306</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8462</v>
+        <v>0.8127147766323024</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7045</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.7688</v>
-      </c>
-      <c r="N8" t="n">
-        <v>6</v>
-      </c>
-      <c r="O8" t="n">
-        <v>42</v>
+        <v>0.8290972830850132</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>42</v>
+      </c>
+      <c r="C9" t="n">
         <v>1462</v>
-      </c>
-      <c r="B9" t="n">
-        <v>182</v>
-      </c>
-      <c r="C9" t="n">
-        <v>237</v>
       </c>
       <c r="D9" t="n">
         <v>419</v>
@@ -3218,45 +3332,36 @@
         <v>209</v>
       </c>
       <c r="F9" t="n">
-        <v>472</v>
+        <v>224</v>
       </c>
       <c r="G9" t="n">
-        <v>2116</v>
+        <v>0.6995215311004784</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6995</v>
+        <v>0.6945368171021378</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6213</v>
+        <v>0.6970202622169248</v>
       </c>
       <c r="J9" t="n">
-        <v>0.6581</v>
+        <v>0.8646062330272857</v>
       </c>
       <c r="K9" t="n">
-        <v>0.8646</v>
+        <v>0.794061757719715</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7104</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.7799</v>
-      </c>
-      <c r="N9" t="n">
-        <v>7</v>
-      </c>
-      <c r="O9" t="n">
-        <v>42</v>
+        <v>0.8278338389153717</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>42</v>
+      </c>
+      <c r="C10" t="n">
         <v>1611</v>
-      </c>
-      <c r="B10" t="n">
-        <v>175</v>
-      </c>
-      <c r="C10" t="n">
-        <v>244</v>
       </c>
       <c r="D10" t="n">
         <v>419</v>
@@ -3265,45 +3370,36 @@
         <v>171</v>
       </c>
       <c r="F10" t="n">
-        <v>414</v>
+        <v>163</v>
       </c>
       <c r="G10" t="n">
-        <v>2200</v>
+        <v>0.7319400272603362</v>
       </c>
       <c r="H10" t="n">
-        <v>0.7319</v>
+        <v>0.7346101231190151</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6592</v>
+        <v>0.7332726445152481</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6936</v>
+        <v>0.878301773006875</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8783</v>
+        <v>0.8301413588691291</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7449</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.8061</v>
-      </c>
-      <c r="N10" t="n">
-        <v>8</v>
-      </c>
-      <c r="O10" t="n">
-        <v>42</v>
+        <v>0.8535427533259099</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>42</v>
+      </c>
+      <c r="C11" t="n">
         <v>1532</v>
-      </c>
-      <c r="B11" t="n">
-        <v>181</v>
-      </c>
-      <c r="C11" t="n">
-        <v>273</v>
       </c>
       <c r="D11" t="n">
         <v>454</v>
@@ -3312,34 +3408,25 @@
         <v>226</v>
       </c>
       <c r="F11" t="n">
-        <v>450</v>
+        <v>176</v>
       </c>
       <c r="G11" t="n">
-        <v>2163</v>
+        <v>0.6925858951175407</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6926</v>
+        <v>0.7086031452358927</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6289</v>
+        <v>0.7005029721079103</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6592</v>
+        <v>0.8611995104039167</v>
       </c>
       <c r="K11" t="n">
-        <v>0.8612</v>
+        <v>0.8135985198889917</v>
       </c>
       <c r="L11" t="n">
-        <v>0.7221</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.7855</v>
-      </c>
-      <c r="N11" t="n">
-        <v>9</v>
-      </c>
-      <c r="O11" t="n">
-        <v>42</v>
+        <v>0.8367225591628017</v>
       </c>
     </row>
   </sheetData>
@@ -3748,34 +3835,34 @@
         <v>0.0199</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6268</v>
+        <v>0.7076</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0203</v>
+        <v>0.0164</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6594</v>
+        <v>0.7015</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0196</v>
+        <v>0.0174</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8619</v>
+        <v>0.8618</v>
       </c>
       <c r="J2" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.8135</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.837</v>
+      </c>
+      <c r="N2" t="n">
         <v>0.0095</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.7205</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.0153</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.7848000000000001</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.0127</v>
       </c>
     </row>
     <row r="3">
@@ -3792,16 +3879,16 @@
         <v>0.02</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6344</v>
+        <v>0.7151999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0174</v>
+        <v>0.0127</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6601</v>
+        <v>0.7013</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0175</v>
+        <v>0.0156</v>
       </c>
       <c r="I3" t="n">
         <v>0.8592</v>
@@ -3810,16 +3897,16 @@
         <v>0.0094</v>
       </c>
       <c r="K3" t="n">
-        <v>0.7296</v>
+        <v>0.8226</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0123</v>
+        <v>0.0067</v>
       </c>
       <c r="M3" t="n">
-        <v>0.7891</v>
+        <v>0.8405</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0104</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="4">
@@ -3836,16 +3923,16 @@
         <v>0.0225</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6322</v>
+        <v>0.7134</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0228</v>
+        <v>0.0203</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6593</v>
+        <v>0.7008</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0218</v>
+        <v>0.0202</v>
       </c>
       <c r="I4" t="n">
         <v>0.859</v>
@@ -3854,16 +3941,16 @@
         <v>0.011</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7282999999999999</v>
+        <v>0.822</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0168</v>
+        <v>0.0144</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7883</v>
+        <v>0.84</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0138</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="5">
@@ -3880,34 +3967,34 @@
         <v>0.0192</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6371</v>
+        <v>0.7179</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0142</v>
+        <v>0.0129</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6615</v>
+        <v>0.7026</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0159</v>
+        <v>0.0152</v>
       </c>
       <c r="I5" t="n">
         <v>0.8593</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0083</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7323</v>
+        <v>0.8252</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0112</v>
+        <v>0.0103</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7907</v>
+        <v>0.8419</v>
       </c>
       <c r="N5" t="n">
-        <v>0.0095</v>
+        <v>0.008200000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3924,16 +4011,16 @@
         <v>0.0184</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6318</v>
+        <v>0.7119</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0177</v>
+        <v>0.0165</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6574</v>
+        <v>0.6983</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0169</v>
+        <v>0.0159</v>
       </c>
       <c r="I6" t="n">
         <v>0.8576</v>
@@ -3942,16 +4029,16 @@
         <v>0.0089</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7287</v>
+        <v>0.8212</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0133</v>
+        <v>0.0129</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7879</v>
+        <v>0.8389</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0106</v>
+        <v>0.0091</v>
       </c>
     </row>
   </sheetData>
@@ -4215,7 +4302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4288,93 +4375,93 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>CoD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6345</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0353</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5488</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0296</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5884</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0303</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8296</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0176</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6626</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0228</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7366</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HX</t>
+          <t>FHx</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7087</v>
+        <v>0.3993</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0639</v>
+        <v>0.2403</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6157</v>
+        <v>0.3732</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0429</v>
+        <v>0.2388</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6582</v>
+        <v>0.3809</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0473</v>
+        <v>0.2339</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8635</v>
+        <v>0.6506</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0332</v>
+        <v>0.2564</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7165</v>
+        <v>0.5473</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0354</v>
+        <v>0.2354</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7824</v>
+        <v>0.5901</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0242</v>
+        <v>0.2391</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LAB</t>
+          <t>Lab</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4384,16 +4471,16 @@
         <v>0.09470000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5091</v>
+        <v>0.5973000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0544</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5486</v>
+        <v>0.5973000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>0.06569999999999999</v>
+        <v>0.0808</v>
       </c>
       <c r="H4" t="n">
         <v>0.8178</v>
@@ -4402,145 +4489,360 @@
         <v>0.0515</v>
       </c>
       <c r="J4" t="n">
-        <v>0.613</v>
+        <v>0.7166</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0562</v>
+        <v>0.052</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6984</v>
+        <v>0.7627</v>
       </c>
       <c r="M4" t="n">
-        <v>0.038</v>
+        <v>0.0431</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>MHx</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6881</v>
+        <v>0.7381</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0374</v>
+        <v>0.06859999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.675</v>
+        <v>0.735</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0324</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6805</v>
+        <v>0.7363</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0236</v>
+        <v>0.068</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8641</v>
+        <v>0.8763</v>
       </c>
       <c r="I5" t="n">
-        <v>0.017</v>
+        <v>0.0354</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7607</v>
+        <v>0.8425</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0327</v>
+        <v>0.0437</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8086</v>
+        <v>0.8588</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0175</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8326</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0476</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7966</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0401</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8139999999999999</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0413</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0.929</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0228</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8459</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0314</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8852</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0231</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.6881</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.7084</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0362</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.6972</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0268</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.8641</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.7982</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.0327</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.8294</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.0185</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SYM</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.5945</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0473</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.6077</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0339</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.6008</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0398</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8107</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0253</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.7514</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.0173</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.7798</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.0173</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.8326</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8494</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0423</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.8408</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0435</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.9018</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.0284</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.9151</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.0229</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>VAX</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B10" t="n">
         <v>0.8512999999999999</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C10" t="n">
         <v>0.0234</v>
       </c>
-      <c r="D7" t="n">
-        <v>0.8384</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.0328</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.8447</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.0265</v>
-      </c>
-      <c r="H7" t="n">
+      <c r="D10" t="n">
+        <v>0.8699</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.0261</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.8604000000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.9352</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I10" t="n">
         <v>0.0112</v>
       </c>
-      <c r="J7" t="n">
-        <v>0.8882</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.0254</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.911</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.0174</v>
+      <c r="J10" t="n">
+        <v>0.9217</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.9283</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.0135</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pDx</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.6964</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.07140000000000001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.6868</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.6907</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0533</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.8584000000000001</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.8001</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.0282</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.8279</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.0246</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sDx</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.7497</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.07240000000000001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.7491</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0564</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.7491</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.06320000000000001</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.8808</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.8554</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.0288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>